<commit_message>
PAUSED (task192, task194): checkpoint, two fix passes mid-rebuild
Continues 8b80059. task192 is rebuilding its checks and figures after re-cutting the
world so the validation sample's coverage and the true rate vary together. task194 is
re-cutting its goldens, chart and metadata while spreading the closed placements'
pre-placement excess so the rival pricings separate on the record.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task194/golden/embed_placement_2027q4.xlsx
+++ b/task194/golden/embed_placement_2027q4.xlsx
@@ -52,16 +52,52 @@
     <t>Complications avoided</t>
   </si>
   <si>
+    <t>41230</t>
+  </si>
+  <si>
+    <t>Alderbrook Orthopaedics</t>
+  </si>
+  <si>
     <t>41220</t>
   </si>
   <si>
     <t>Alderbrook General Surgery</t>
   </si>
   <si>
-    <t>41230</t>
-  </si>
-  <si>
-    <t>Alderbrook Orthopaedics</t>
+    <t>41420</t>
+  </si>
+  <si>
+    <t>Marrowfield General Medicine</t>
+  </si>
+  <si>
+    <t>41310</t>
+  </si>
+  <si>
+    <t>Stonecreek General Medicine</t>
+  </si>
+  <si>
+    <t>41330</t>
+  </si>
+  <si>
+    <t>Stonecreek Vascular Surgery</t>
+  </si>
+  <si>
+    <t>41240</t>
+  </si>
+  <si>
+    <t>Alderbrook Respiratory Medicine</t>
+  </si>
+  <si>
+    <t>41520</t>
+  </si>
+  <si>
+    <t>Marrowfield Surgical Services</t>
+  </si>
+  <si>
+    <t>41510</t>
+  </si>
+  <si>
+    <t>Carrowdean General Medicine</t>
   </si>
   <si>
     <t>41210</t>
@@ -70,40 +106,10 @@
     <t>Alderbrook General Medicine</t>
   </si>
   <si>
-    <t>41420</t>
-  </si>
-  <si>
-    <t>Marrowfield General Medicine</t>
-  </si>
-  <si>
-    <t>41310</t>
-  </si>
-  <si>
-    <t>Stonecreek General Medicine</t>
-  </si>
-  <si>
-    <t>41330</t>
-  </si>
-  <si>
-    <t>Stonecreek Vascular Surgery</t>
-  </si>
-  <si>
-    <t>41510</t>
-  </si>
-  <si>
-    <t>Carrowdean General Medicine</t>
-  </si>
-  <si>
-    <t>41240</t>
-  </si>
-  <si>
-    <t>Alderbrook Respiratory Medicine</t>
-  </si>
-  <si>
-    <t>41520</t>
-  </si>
-  <si>
-    <t>Marrowfield Surgical Services</t>
+    <t>41320</t>
+  </si>
+  <si>
+    <t>Stonecreek General Surgery</t>
   </si>
   <si>
     <t>41410</t>
@@ -118,22 +124,16 @@
     <t>Stonecreek Renal Medicine</t>
   </si>
   <si>
-    <t>41320</t>
-  </si>
-  <si>
-    <t>Stonecreek General Surgery</t>
-  </si>
-  <si>
     <t>Recommendation</t>
   </si>
   <si>
+    <t>Alderbrook Orthopaedics (41230)</t>
+  </si>
+  <si>
+    <t>Closest unit</t>
+  </si>
+  <si>
     <t>Alderbrook General Surgery (41220)</t>
-  </si>
-  <si>
-    <t>Closest unit</t>
-  </si>
-  <si>
-    <t>Alderbrook Orthopaedics (41230)</t>
   </si>
   <si>
     <t>Complications avoided there</t>
@@ -750,16 +750,16 @@
         <v>9</v>
       </c>
       <c r="C5" s="4">
-        <v>3560</v>
+        <v>2305</v>
       </c>
       <c r="D5" s="5">
-        <v>276.1</v>
+        <v>199.2</v>
       </c>
       <c r="E5" s="6">
-        <v>1.19</v>
+        <v>1.24</v>
       </c>
       <c r="F5" s="4">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -770,16 +770,16 @@
         <v>11</v>
       </c>
       <c r="C6" s="4">
-        <v>2305</v>
+        <v>3560</v>
       </c>
       <c r="D6" s="5">
-        <v>199.2</v>
+        <v>276.1</v>
       </c>
       <c r="E6" s="6">
-        <v>1.24</v>
+        <v>1.12</v>
       </c>
       <c r="F6" s="4">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -790,16 +790,16 @@
         <v>13</v>
       </c>
       <c r="C7" s="4">
-        <v>2077</v>
+        <v>1162</v>
       </c>
       <c r="D7" s="5">
-        <v>169.7</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="E7" s="6">
-        <v>1.08</v>
+        <v>1.25</v>
       </c>
       <c r="F7" s="4">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -810,16 +810,16 @@
         <v>15</v>
       </c>
       <c r="C8" s="4">
-        <v>1162</v>
+        <v>1362</v>
       </c>
       <c r="D8" s="5">
-        <v>92.09999999999999</v>
+        <v>108.8</v>
       </c>
       <c r="E8" s="6">
-        <v>1.1</v>
+        <v>1.16</v>
       </c>
       <c r="F8" s="4">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -830,16 +830,16 @@
         <v>17</v>
       </c>
       <c r="C9" s="4">
-        <v>1364</v>
+        <v>506</v>
       </c>
       <c r="D9" s="5">
-        <v>109</v>
+        <v>50.5</v>
       </c>
       <c r="E9" s="6">
-        <v>1.07</v>
+        <v>1.31</v>
       </c>
       <c r="F9" s="4">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -850,16 +850,16 @@
         <v>19</v>
       </c>
       <c r="C10" s="4">
-        <v>506</v>
+        <v>1257</v>
       </c>
       <c r="D10" s="5">
-        <v>50.5</v>
+        <v>118.1</v>
       </c>
       <c r="E10" s="6">
         <v>1.1</v>
       </c>
       <c r="F10" s="4">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -870,16 +870,16 @@
         <v>21</v>
       </c>
       <c r="C11" s="4">
-        <v>466</v>
+        <v>779</v>
       </c>
       <c r="D11" s="5">
-        <v>38.5</v>
+        <v>59.1</v>
       </c>
       <c r="E11" s="6">
-        <v>0.95</v>
+        <v>1.13</v>
       </c>
       <c r="F11" s="4">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -890,16 +890,16 @@
         <v>23</v>
       </c>
       <c r="C12" s="4">
-        <v>1257</v>
+        <v>466</v>
       </c>
       <c r="D12" s="5">
-        <v>118.1</v>
+        <v>38.5</v>
       </c>
       <c r="E12" s="6">
-        <v>0.98</v>
+        <v>1.19</v>
       </c>
       <c r="F12" s="4">
-        <v>-1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -910,16 +910,16 @@
         <v>25</v>
       </c>
       <c r="C13" s="4">
-        <v>779</v>
+        <v>1979</v>
       </c>
       <c r="D13" s="5">
-        <v>59.1</v>
+        <v>161.7</v>
       </c>
       <c r="E13" s="6">
-        <v>0.91</v>
+        <v>1.04</v>
       </c>
       <c r="F13" s="4">
-        <v>-3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -930,16 +930,16 @@
         <v>27</v>
       </c>
       <c r="C14" s="4">
-        <v>734</v>
+        <v>1469</v>
       </c>
       <c r="D14" s="5">
-        <v>61.5</v>
+        <v>113.9</v>
       </c>
       <c r="E14" s="6">
-        <v>0.88</v>
+        <v>1.05</v>
       </c>
       <c r="F14" s="4">
-        <v>-4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -950,16 +950,16 @@
         <v>29</v>
       </c>
       <c r="C15" s="4">
-        <v>652</v>
+        <v>734</v>
       </c>
       <c r="D15" s="5">
-        <v>51.2</v>
+        <v>61.5</v>
       </c>
       <c r="E15" s="6">
-        <v>0.84</v>
+        <v>1.09</v>
       </c>
       <c r="F15" s="4">
-        <v>-5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -970,16 +970,16 @@
         <v>31</v>
       </c>
       <c r="C16" s="4">
-        <v>1469</v>
+        <v>717</v>
       </c>
       <c r="D16" s="5">
-        <v>113.9</v>
+        <v>56.3</v>
       </c>
       <c r="E16" s="6">
-        <v>0.93</v>
+        <v>1.06</v>
       </c>
       <c r="F16" s="4">
-        <v>-5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -995,7 +995,7 @@
         <v>7</v>
       </c>
       <c r="B19">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -1011,7 +1011,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1019,7 +1019,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -1070,10 +1070,10 @@
         <v>46925</v>
       </c>
       <c r="C5" s="4">
-        <v>4841</v>
+        <v>4893</v>
       </c>
       <c r="D5" s="5">
-        <v>105.2</v>
+        <v>106.3</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1084,10 +1084,10 @@
         <v>29194</v>
       </c>
       <c r="C6" s="4">
-        <v>3626</v>
+        <v>3856</v>
       </c>
       <c r="D6" s="5">
-        <v>126.8</v>
+        <v>134.8</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1098,10 +1098,10 @@
         <v>23903</v>
       </c>
       <c r="C7" s="4">
-        <v>2522</v>
+        <v>2650</v>
       </c>
       <c r="D7" s="5">
-        <v>113.1</v>
+        <v>118.8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1112,10 +1112,10 @@
         <v>2340</v>
       </c>
       <c r="C8" s="4">
-        <v>191</v>
+        <v>240</v>
       </c>
       <c r="D8" s="5">
-        <v>91.09999999999999</v>
+        <v>114.5</v>
       </c>
     </row>
   </sheetData>
@@ -1312,10 +1312,10 @@
         <v>70</v>
       </c>
       <c r="C5" s="4">
-        <v>2742</v>
+        <v>2843</v>
       </c>
       <c r="D5" s="4">
-        <v>1299</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1326,10 +1326,10 @@
         <v>72</v>
       </c>
       <c r="C6" s="4">
-        <v>1839</v>
+        <v>1906</v>
       </c>
       <c r="D6" s="4">
-        <v>859</v>
+        <v>931</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1340,10 +1340,10 @@
         <v>74</v>
       </c>
       <c r="C7" s="4">
-        <v>1618</v>
+        <v>1681</v>
       </c>
       <c r="D7" s="4">
-        <v>775</v>
+        <v>845</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1354,10 +1354,10 @@
         <v>76</v>
       </c>
       <c r="C8" s="4">
-        <v>1854</v>
+        <v>1908</v>
       </c>
       <c r="D8" s="4">
-        <v>930</v>
+        <v>978</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1368,10 +1368,10 @@
         <v>78</v>
       </c>
       <c r="C9" s="4">
-        <v>2192</v>
+        <v>2269</v>
       </c>
       <c r="D9" s="4">
-        <v>1022</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1382,10 +1382,10 @@
         <v>80</v>
       </c>
       <c r="C10" s="4">
-        <v>2178</v>
+        <v>2241</v>
       </c>
       <c r="D10" s="4">
-        <v>1062</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1396,10 +1396,10 @@
         <v>82</v>
       </c>
       <c r="C11" s="4">
-        <v>1093</v>
+        <v>1100</v>
       </c>
       <c r="D11" s="4">
-        <v>553</v>
+        <v>566</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1410,10 +1410,10 @@
         <v>84</v>
       </c>
       <c r="C12" s="4">
-        <v>1225</v>
+        <v>1243</v>
       </c>
       <c r="D12" s="4">
-        <v>585</v>
+        <v>605</v>
       </c>
     </row>
   </sheetData>

</xml_diff>